<commit_message>
Add evaluation-list PDF export and align Excel output with system scores, N/A totals, and grade colors.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/exercise_store/رياح الصحراء 2026_20_files/evaluation_list_xlsx/ul_ew/ibn_5955.xlsx
+++ b/exercise_store/رياح الصحراء 2026_20_files/evaluation_list_xlsx/ul_ew/ibn_5955.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20397"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B8465A-689E-4A62-9761-3509B16622D6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570"/>
   </bookViews>
   <sheets>
     <sheet name="قائمة التقييم" sheetId="2" r:id="rId1"/>
@@ -17,7 +16,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'قائمة التقييم'!$A$1:$J$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'قائمة التقييم'!$4:$4</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="189">
   <si>
     <t>عناصــــــر التقييـــــم</t>
   </si>
@@ -853,7 +852,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-10C0000]d\ mmmm\ yyyy;@"/>
   </numFmts>
@@ -861,7 +860,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -890,7 +889,7 @@
     <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -926,7 +925,7 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -939,7 +938,7 @@
     <font>
       <b/>
       <sz val="12"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1382,6 +1381,64 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
       <protection locked="0"/>
@@ -1402,6 +1459,23 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="2"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="top" wrapText="1" readingOrder="2"/>
       <protection locked="0"/>
@@ -1423,87 +1497,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="20">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -1554,26 +1553,6 @@
           <bgColor rgb="FF00B0F0"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -1972,60 +1951,60 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE1D0DF2-5DCE-4624-B909-68D4EC5F2664}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J21"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="5.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="9" style="1"/>
-    <col min="4" max="4" width="28.125" style="1" customWidth="1"/>
-    <col min="5" max="7" width="9.25" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.25" style="3" customWidth="1"/>
-    <col min="9" max="9" width="9.25" style="1" customWidth="1"/>
-    <col min="10" max="10" width="15.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.140625" style="1" customWidth="1"/>
+    <col min="5" max="7" width="9.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.28515625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="9.28515625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" style="1" customWidth="1"/>
     <col min="11" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="58" t="s">
+    <row r="1" spans="1:10" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="28" t="s">
         <v>188</v>
       </c>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58"/>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-    </row>
-    <row r="2" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+    </row>
+    <row r="2" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7"/>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="47" t="s">
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47" t="s">
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="J2" s="48"/>
-    </row>
-    <row r="3" spans="1:10" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J2" s="38"/>
+    </row>
+    <row r="3" spans="1:10" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
-      <c r="B3" s="41"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
       <c r="E3" s="8" t="s">
         <v>3</v>
       </c>
@@ -2038,16 +2017,16 @@
       <c r="H3" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="49"/>
-      <c r="J3" s="50"/>
-    </row>
-    <row r="4" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="I3" s="39"/>
+      <c r="J3" s="40"/>
+    </row>
+    <row r="4" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
       <c r="E4" s="23" t="s">
         <v>14</v>
       </c>
@@ -2060,12 +2039,12 @@
       <c r="H4" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="51" t="s">
+      <c r="I4" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="52"/>
-    </row>
-    <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J4" s="42"/>
+    </row>
+    <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="27" t="s">
         <v>176</v>
@@ -2075,21 +2054,13 @@
       <c r="E5" s="6">
         <v>5</v>
       </c>
-      <c r="F5" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G5" s="25" t="str">
-        <f>IFERROR(F5/E5,"")</f>
-        <v/>
-      </c>
-      <c r="H5" s="26" t="str">
-        <f>_xlfn.IFS(F5="أدخل العلامة","",F5="لا ينطبق","تم الإلغاء",G5&gt;=90%,"ممتاز",G5&gt;=80%,"جيد جداً",G5&gt;=70%,"جيد",G5&gt;=60%,"مقبول",G5&lt;60%,"راسب")</f>
-        <v/>
-      </c>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-    </row>
-    <row r="6" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F5" s="22"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="43"/>
+      <c r="J5" s="43"/>
+    </row>
+    <row r="6" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="27" t="s">
         <v>177</v>
@@ -2099,21 +2070,13 @@
       <c r="E6" s="6">
         <v>5</v>
       </c>
-      <c r="F6" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G6" s="25" t="str">
-        <f>IFERROR(F6/E6,"")</f>
-        <v/>
-      </c>
-      <c r="H6" s="26" t="str">
-        <f>_xlfn.IFS(F6="أدخل العلامة","",F6="لا ينطبق","تم الإلغاء",G6&gt;=90%,"ممتاز",G6&gt;=80%,"جيد جداً",G6&gt;=70%,"جيد",G6&gt;=60%,"مقبول",G6&lt;60%,"راسب")</f>
-        <v/>
-      </c>
-      <c r="I6" s="28"/>
-      <c r="J6" s="28"/>
-    </row>
-    <row r="7" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F6" s="22"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="43"/>
+    </row>
+    <row r="7" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
       <c r="B7" s="27" t="s">
         <v>186</v>
@@ -2123,21 +2086,13 @@
       <c r="E7" s="6">
         <v>5</v>
       </c>
-      <c r="F7" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G7" s="25" t="str">
-        <f t="shared" ref="G7:G16" si="0">IFERROR(F7/E7,"")</f>
-        <v/>
-      </c>
-      <c r="H7" s="26" t="str">
-        <f t="shared" ref="H7:H16" si="1">_xlfn.IFS(F7="أدخل العلامة","",F7="لا ينطبق","تم الإلغاء",G7&gt;=90%,"ممتاز",G7&gt;=80%,"جيد جداً",G7&gt;=70%,"جيد",G7&gt;=60%,"مقبول",G7&lt;60%,"راسب")</f>
-        <v/>
-      </c>
-      <c r="I7" s="28"/>
-      <c r="J7" s="28"/>
-    </row>
-    <row r="8" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F7" s="22"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="26"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+    </row>
+    <row r="8" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
       <c r="B8" s="27" t="s">
         <v>178</v>
@@ -2147,21 +2102,13 @@
       <c r="E8" s="6">
         <v>5</v>
       </c>
-      <c r="F8" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G8" s="25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H8" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I8" s="28"/>
-      <c r="J8" s="28"/>
-    </row>
-    <row r="9" spans="1:10" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F8" s="22"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+    </row>
+    <row r="9" spans="1:10" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="27" t="s">
         <v>179</v>
@@ -2171,21 +2118,13 @@
       <c r="E9" s="6">
         <v>5</v>
       </c>
-      <c r="F9" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G9" s="25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H9" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-    </row>
-    <row r="10" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F9" s="22"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="43"/>
+    </row>
+    <row r="10" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7"/>
       <c r="B10" s="27" t="s">
         <v>180</v>
@@ -2195,21 +2134,13 @@
       <c r="E10" s="6">
         <v>5</v>
       </c>
-      <c r="F10" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G10" s="25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H10" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-    </row>
-    <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F10" s="22"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="43"/>
+      <c r="J10" s="43"/>
+    </row>
+    <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
       <c r="B11" s="27" t="s">
         <v>181</v>
@@ -2219,21 +2150,13 @@
       <c r="E11" s="6">
         <v>5</v>
       </c>
-      <c r="F11" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G11" s="25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H11" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I11" s="28"/>
-      <c r="J11" s="28"/>
-    </row>
-    <row r="12" spans="1:10" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F11" s="22"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="43"/>
+      <c r="J11" s="43"/>
+    </row>
+    <row r="12" spans="1:10" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
       <c r="B12" s="27" t="s">
         <v>187</v>
@@ -2243,21 +2166,13 @@
       <c r="E12" s="6">
         <v>5</v>
       </c>
-      <c r="F12" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G12" s="25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H12" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
-    </row>
-    <row r="13" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F12" s="22"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="43"/>
+      <c r="J12" s="43"/>
+    </row>
+    <row r="13" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="27" t="s">
         <v>182</v>
@@ -2267,21 +2182,13 @@
       <c r="E13" s="6">
         <v>5</v>
       </c>
-      <c r="F13" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G13" s="25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H13" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
-    </row>
-    <row r="14" spans="1:10" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F13" s="22"/>
+      <c r="G13" s="25"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43"/>
+    </row>
+    <row r="14" spans="1:10" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
       <c r="B14" s="27" t="s">
         <v>183</v>
@@ -2291,21 +2198,13 @@
       <c r="E14" s="6">
         <v>5</v>
       </c>
-      <c r="F14" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G14" s="25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H14" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
-    </row>
-    <row r="15" spans="1:10" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F14" s="22"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43"/>
+    </row>
+    <row r="15" spans="1:10" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
       <c r="B15" s="27" t="s">
         <v>184</v>
@@ -2315,21 +2214,13 @@
       <c r="E15" s="6">
         <v>5</v>
       </c>
-      <c r="F15" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G15" s="25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H15" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
-    </row>
-    <row r="16" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F15" s="22"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="43"/>
+      <c r="J15" s="43"/>
+    </row>
+    <row r="16" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="27" t="s">
         <v>185</v>
@@ -2339,107 +2230,90 @@
       <c r="E16" s="6">
         <v>5</v>
       </c>
-      <c r="F16" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="G16" s="25" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="H16" s="26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="I16" s="28"/>
-      <c r="J16" s="28"/>
-    </row>
-    <row r="17" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F16" s="22"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43"/>
+    </row>
+    <row r="17" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
-      <c r="B17" s="29" t="s">
+      <c r="B17" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="24">
-        <f>SUM(E5:E16)</f>
-        <v>60</v>
-      </c>
+      <c r="C17" s="45"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="24"/>
       <c r="F17" s="24">
         <f>SUM(F5:F16)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="55"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="56"/>
-      <c r="J17" s="57"/>
-    </row>
-    <row r="18" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="G17" s="50"/>
+      <c r="H17" s="51"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="52"/>
+    </row>
+    <row r="18" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="43">
-        <f>F17/E17/100*100</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="43"/>
-      <c r="G18" s="43"/>
-      <c r="H18" s="43"/>
-      <c r="I18" s="43"/>
-      <c r="J18" s="44"/>
-    </row>
-    <row r="19" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+      <c r="I18" s="33"/>
+      <c r="J18" s="34"/>
+    </row>
+    <row r="19" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="46" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="37" t="str">
-        <f>_xlfn.IFS(E18&gt;=90%,"ممتاز",E18&gt;=80%,"جيد جداً",E18&gt;=70%,"جيد",E18&gt;=60%,"مقبول",E18&lt;60%,"راسب")</f>
-        <v>راسب</v>
-      </c>
-      <c r="F19" s="37"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="37"/>
-      <c r="I19" s="37"/>
-      <c r="J19" s="38"/>
-    </row>
-    <row r="20" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="33" t="s">
+      <c r="C19" s="47"/>
+      <c r="D19" s="47"/>
+      <c r="E19" s="57"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="57"/>
+      <c r="I19" s="57"/>
+      <c r="J19" s="58"/>
+    </row>
+    <row r="20" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="53" t="s">
         <v>170</v>
       </c>
-      <c r="C20" s="33"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="53" t="s">
+      <c r="C20" s="53"/>
+      <c r="D20" s="53"/>
+      <c r="E20" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="F20" s="53"/>
-      <c r="G20" s="35" t="s">
+      <c r="F20" s="48"/>
+      <c r="G20" s="55" t="s">
         <v>55</v>
       </c>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-    </row>
-    <row r="21" spans="1:10" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H20" s="55"/>
+      <c r="I20" s="55"/>
+      <c r="J20" s="55"/>
+    </row>
+    <row r="21" spans="1:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
-      <c r="B21" s="34"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="54" t="s">
+      <c r="B21" s="54"/>
+      <c r="C21" s="54"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="49" t="s">
         <v>49</v>
       </c>
-      <c r="F21" s="54"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="36"/>
+      <c r="F21" s="49"/>
+      <c r="G21" s="56"/>
+      <c r="H21" s="56"/>
+      <c r="I21" s="56"/>
+      <c r="J21" s="56"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0"/>
   <mergeCells count="41">
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="E21:F21"/>
@@ -2449,6 +2323,14 @@
     <mergeCell ref="G20:J20"/>
     <mergeCell ref="G21:J21"/>
     <mergeCell ref="E19:J19"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
     <mergeCell ref="B1:J1"/>
     <mergeCell ref="B2:D3"/>
     <mergeCell ref="E18:J18"/>
@@ -2460,67 +2342,59 @@
     <mergeCell ref="I5:J5"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="I12:J12"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
   </mergeCells>
   <conditionalFormatting sqref="E19">
-    <cfRule type="expression" dxfId="23" priority="57">
+    <cfRule type="expression" dxfId="19" priority="57">
       <formula>$E19="راسب"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E19:J19">
-    <cfRule type="expression" dxfId="22" priority="58">
+    <cfRule type="expression" dxfId="18" priority="58">
       <formula>$E19="مقبول"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="59">
+    <cfRule type="expression" dxfId="17" priority="59">
       <formula>$E19="جيد"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="60">
+    <cfRule type="expression" dxfId="16" priority="60">
       <formula>$E19="جيد جداً"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="61">
+    <cfRule type="expression" dxfId="15" priority="61">
       <formula>$E19="ممتاز"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5 H7:H16">
-    <cfRule type="containsText" dxfId="18" priority="39" operator="containsText" text="ممتاز">
+    <cfRule type="containsText" dxfId="14" priority="39" operator="containsText" text="ممتاز">
       <formula>NOT(ISERROR(SEARCH("ممتاز",H5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="40" operator="containsText" text="جيد جداً">
+    <cfRule type="containsText" dxfId="13" priority="40" operator="containsText" text="جيد جداً">
       <formula>NOT(ISERROR(SEARCH("جيد جداً",H5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="41" operator="containsText" text="جيد">
+    <cfRule type="containsText" dxfId="12" priority="41" operator="containsText" text="جيد">
       <formula>NOT(ISERROR(SEARCH("جيد",H5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="42" operator="containsText" text="مقبول">
+    <cfRule type="containsText" dxfId="11" priority="42" operator="containsText" text="مقبول">
       <formula>NOT(ISERROR(SEARCH("مقبول",H5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="43" operator="containsText" text="راسب">
+    <cfRule type="containsText" dxfId="10" priority="43" operator="containsText" text="راسب">
       <formula>NOT(ISERROR(SEARCH("راسب",H5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5 H7:H16">
-    <cfRule type="containsText" dxfId="13" priority="38" operator="containsText" text="أدخل العلامة">
+    <cfRule type="containsText" dxfId="9" priority="38" operator="containsText" text="أدخل العلامة">
       <formula>NOT(ISERROR(SEARCH("أدخل العلامة",H5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2563,7 +2437,7 @@
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="69" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="75" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"-,Bold"&amp;12&amp;Uسري للغاية</oddHeader>
     <oddFooter>&amp;C&amp;"-,Bold"&amp;P&amp;"-,Regular"
@@ -2572,13 +2446,13 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5A7ADC9F-6098-4415-8DD4-849A148D02E3}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>'بيانات التقييم'!$A$111:$A$133</xm:f>
           </x14:formula1>
           <xm:sqref>F5:F16</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BD8CB5A2-5F32-4EAD-A63C-382D3B90B847}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>'بيانات التقييم'!$A$198:$A$286</xm:f>
           </x14:formula1>
@@ -2591,18 +2465,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E0E097-B5B4-4A62-8BA3-2420E658D743}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:I338"/>
-  <sheetFormatPr defaultRowHeight="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="59.875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="42.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="59.85546875" style="1" customWidth="1"/>
     <col min="4" max="9" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>53</v>
       </c>
@@ -2610,7 +2484,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>31</v>
       </c>
@@ -2618,7 +2492,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
@@ -2626,7 +2500,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>32</v>
       </c>
@@ -2634,7 +2508,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -2642,7 +2516,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
@@ -2650,7 +2524,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
@@ -2658,7 +2532,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>36</v>
       </c>
@@ -2666,7 +2540,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
@@ -2674,7 +2548,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>38</v>
       </c>
@@ -2682,7 +2556,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>39</v>
       </c>
@@ -2690,7 +2564,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>40</v>
       </c>
@@ -2698,7 +2572,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>41</v>
       </c>
@@ -2706,7 +2580,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>42</v>
       </c>
@@ -2714,7 +2588,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>43</v>
       </c>
@@ -2722,7 +2596,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>6</v>
       </c>
@@ -2730,7 +2604,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>23</v>
       </c>
@@ -2738,7 +2612,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>44</v>
       </c>
@@ -2746,7 +2620,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>45</v>
       </c>
@@ -2754,7 +2628,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
@@ -2762,7 +2636,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>47</v>
       </c>
@@ -2770,7 +2644,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>7</v>
       </c>
@@ -2778,7 +2652,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>8</v>
       </c>
@@ -2786,7 +2660,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>11</v>
       </c>
@@ -2794,7 +2668,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -2802,7 +2676,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
@@ -2810,7 +2684,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>9</v>
       </c>
@@ -2818,7 +2692,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -2826,7 +2700,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -2834,7 +2708,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -2842,7 +2716,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -2850,28 +2724,28 @@
         <v>175</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C32" s="15"/>
     </row>
-    <row r="33" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C33" s="15"/>
     </row>
-    <row r="34" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>30</v>
       </c>
       <c r="C34" s="15"/>
     </row>
-    <row r="35" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14"/>
     </row>
-    <row r="36" spans="1:9" s="13" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" s="13" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11"/>
       <c r="B36" s="12"/>
       <c r="C36" s="12"/>
@@ -2882,285 +2756,285 @@
       <c r="H36" s="12"/>
       <c r="I36" s="12"/>
     </row>
-    <row r="37" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="9">
         <v>45931</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="9">
         <v>45932</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="9">
         <v>45933</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="9">
         <v>45934</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="9">
         <v>45935</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="9">
         <v>45936</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="9">
         <v>45937</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="9">
         <v>45938</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="9">
         <v>45939</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="9">
         <v>45940</v>
       </c>
     </row>
-    <row r="49" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="9">
         <v>45941</v>
       </c>
     </row>
-    <row r="50" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="9">
         <v>45942</v>
       </c>
     </row>
-    <row r="51" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="9">
         <v>45943</v>
       </c>
     </row>
-    <row r="52" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9">
         <v>45944</v>
       </c>
     </row>
-    <row r="53" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="9">
         <v>45945</v>
       </c>
     </row>
-    <row r="54" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="9">
         <v>45946</v>
       </c>
     </row>
-    <row r="55" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="9">
         <v>45947</v>
       </c>
     </row>
-    <row r="56" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="9">
         <v>45948</v>
       </c>
     </row>
-    <row r="57" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="9">
         <v>45949</v>
       </c>
     </row>
-    <row r="58" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="9">
         <v>45950</v>
       </c>
     </row>
-    <row r="59" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="9">
         <v>45951</v>
       </c>
     </row>
-    <row r="60" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="9">
         <v>45952</v>
       </c>
     </row>
-    <row r="61" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="9">
         <v>45953</v>
       </c>
     </row>
-    <row r="62" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="9">
         <v>45954</v>
       </c>
     </row>
-    <row r="63" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="9">
         <v>45955</v>
       </c>
     </row>
-    <row r="64" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="9">
         <v>45956</v>
       </c>
     </row>
-    <row r="65" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="9">
         <v>45957</v>
       </c>
     </row>
-    <row r="66" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="9">
         <v>45958</v>
       </c>
     </row>
-    <row r="67" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="9">
         <v>45959</v>
       </c>
     </row>
-    <row r="68" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="9">
         <v>45960</v>
       </c>
     </row>
-    <row r="69" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="9">
         <v>45961</v>
       </c>
     </row>
-    <row r="70" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="9"/>
     </row>
-    <row r="71" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="9"/>
     </row>
-    <row r="72" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="9"/>
     </row>
-    <row r="73" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="9"/>
     </row>
-    <row r="74" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="9"/>
     </row>
-    <row r="75" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="9"/>
     </row>
-    <row r="76" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="9"/>
     </row>
-    <row r="77" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="9"/>
     </row>
-    <row r="78" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A78" s="9"/>
     </row>
-    <row r="79" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="9"/>
     </row>
-    <row r="80" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="9"/>
     </row>
-    <row r="81" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="9"/>
     </row>
-    <row r="82" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="9"/>
     </row>
-    <row r="83" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="9"/>
     </row>
-    <row r="84" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="9"/>
     </row>
-    <row r="85" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="9"/>
     </row>
-    <row r="86" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="9"/>
     </row>
-    <row r="87" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="9"/>
     </row>
-    <row r="88" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="9"/>
     </row>
-    <row r="89" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="9"/>
     </row>
-    <row r="90" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="9"/>
     </row>
-    <row r="91" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="9"/>
     </row>
-    <row r="92" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="9"/>
     </row>
-    <row r="93" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="9"/>
     </row>
-    <row r="94" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="9"/>
     </row>
-    <row r="95" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="9"/>
     </row>
-    <row r="96" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="9"/>
     </row>
-    <row r="97" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="9"/>
     </row>
-    <row r="98" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="9"/>
     </row>
-    <row r="99" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="9"/>
     </row>
-    <row r="100" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="9"/>
     </row>
-    <row r="101" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="9"/>
     </row>
-    <row r="102" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="9"/>
     </row>
-    <row r="103" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="9"/>
     </row>
-    <row r="104" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="9"/>
     </row>
-    <row r="105" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="9"/>
     </row>
-    <row r="106" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A106" s="9"/>
     </row>
-    <row r="107" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="10"/>
     </row>
-    <row r="108" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="10"/>
     </row>
-    <row r="109" spans="1:9" s="13" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:9" s="13" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="11"/>
       <c r="B109" s="12"/>
       <c r="C109" s="12"/>
@@ -3171,1124 +3045,1124 @@
       <c r="H109" s="12"/>
       <c r="I109" s="12"/>
     </row>
-    <row r="110" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="111" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A113" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2">
         <v>0.25</v>
       </c>
     </row>
-    <row r="115" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A115" s="2">
         <v>0.5</v>
       </c>
     </row>
-    <row r="116" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="2">
         <v>0.75</v>
       </c>
     </row>
-    <row r="117" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>1.25</v>
       </c>
     </row>
-    <row r="119" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2">
         <v>1.5</v>
       </c>
     </row>
-    <row r="120" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2">
         <v>1.75</v>
       </c>
     </row>
-    <row r="121" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="122" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2">
         <v>2.25</v>
       </c>
     </row>
-    <row r="123" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="2">
         <v>2.5</v>
       </c>
     </row>
-    <row r="124" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A124" s="2">
         <v>2.75</v>
       </c>
     </row>
-    <row r="125" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="126" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A126" s="2">
         <v>3.25</v>
       </c>
     </row>
-    <row r="127" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" s="2">
         <v>3.5</v>
       </c>
     </row>
-    <row r="128" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="2">
         <v>3.75</v>
       </c>
     </row>
-    <row r="129" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="130" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2">
         <v>4.25</v>
       </c>
     </row>
-    <row r="131" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2">
         <v>4.5</v>
       </c>
     </row>
-    <row r="132" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2">
         <v>4.75</v>
       </c>
     </row>
-    <row r="133" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A133" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="134" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2">
         <v>5.25</v>
       </c>
     </row>
-    <row r="135" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A135" s="2">
         <v>5.5</v>
       </c>
     </row>
-    <row r="136" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A136" s="2">
         <v>5.75</v>
       </c>
     </row>
-    <row r="137" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A137" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="138" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A138" s="2">
         <v>6.25</v>
       </c>
     </row>
-    <row r="139" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A139" s="2">
         <v>6.5</v>
       </c>
     </row>
-    <row r="140" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A140" s="2">
         <v>6.75</v>
       </c>
     </row>
-    <row r="141" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A141" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="142" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A142" s="2">
         <v>7.25</v>
       </c>
     </row>
-    <row r="143" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A143" s="2">
         <v>7.5</v>
       </c>
     </row>
-    <row r="144" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A144" s="2">
         <v>7.75</v>
       </c>
     </row>
-    <row r="145" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A145" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="146" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A146" s="2">
         <v>8.25</v>
       </c>
     </row>
-    <row r="147" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A147" s="2">
         <v>8.5</v>
       </c>
     </row>
-    <row r="148" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A148" s="2">
         <v>8.75</v>
       </c>
     </row>
-    <row r="149" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A149" s="2">
         <v>9</v>
       </c>
     </row>
-    <row r="150" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A150" s="2">
         <v>9.25</v>
       </c>
     </row>
-    <row r="151" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A151" s="2">
         <v>9.5</v>
       </c>
     </row>
-    <row r="152" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A152" s="2">
         <v>9.75</v>
       </c>
     </row>
-    <row r="153" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A153" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="154" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2">
         <v>10.25</v>
       </c>
     </row>
-    <row r="155" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A155" s="2">
         <v>10.5</v>
       </c>
     </row>
-    <row r="156" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A156" s="2">
         <v>10.75</v>
       </c>
     </row>
-    <row r="157" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A157" s="2">
         <v>11</v>
       </c>
     </row>
-    <row r="158" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A158" s="2">
         <v>11.25</v>
       </c>
     </row>
-    <row r="159" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A159" s="2">
         <v>11.5</v>
       </c>
     </row>
-    <row r="160" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A160" s="2">
         <v>11.75</v>
       </c>
     </row>
-    <row r="161" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A161" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="162" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A162" s="2">
         <v>12.25</v>
       </c>
     </row>
-    <row r="163" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A163" s="2">
         <v>12.5</v>
       </c>
     </row>
-    <row r="164" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A164" s="2">
         <v>12.75</v>
       </c>
     </row>
-    <row r="165" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A165" s="2">
         <v>13</v>
       </c>
     </row>
-    <row r="166" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A166" s="2">
         <v>13.25</v>
       </c>
     </row>
-    <row r="167" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A167" s="2">
         <v>13.5</v>
       </c>
     </row>
-    <row r="168" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A168" s="2">
         <v>13.75</v>
       </c>
     </row>
-    <row r="169" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A169" s="2">
         <v>14</v>
       </c>
     </row>
-    <row r="170" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A170" s="2">
         <v>14.25</v>
       </c>
     </row>
-    <row r="171" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A171" s="2">
         <v>14.5</v>
       </c>
     </row>
-    <row r="172" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A172" s="2">
         <v>14.75</v>
       </c>
     </row>
-    <row r="173" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A173" s="2">
         <v>15</v>
       </c>
     </row>
-    <row r="174" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A174" s="2">
         <v>15.25</v>
       </c>
     </row>
-    <row r="175" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A175" s="2">
         <v>15.5</v>
       </c>
     </row>
-    <row r="176" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A176" s="2">
         <v>15.75</v>
       </c>
     </row>
-    <row r="177" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A177" s="2">
         <v>16</v>
       </c>
     </row>
-    <row r="178" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A178" s="2">
         <v>16.25</v>
       </c>
     </row>
-    <row r="179" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A179" s="2">
         <v>16.5</v>
       </c>
     </row>
-    <row r="180" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A180" s="2">
         <v>16.75</v>
       </c>
     </row>
-    <row r="181" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A181" s="2">
         <v>17</v>
       </c>
     </row>
-    <row r="182" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A182" s="2">
         <v>17.25</v>
       </c>
     </row>
-    <row r="183" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A183" s="2">
         <v>17.5</v>
       </c>
     </row>
-    <row r="184" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A184" s="2">
         <v>17.75</v>
       </c>
     </row>
-    <row r="185" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A185" s="2">
         <v>18</v>
       </c>
     </row>
-    <row r="186" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A186" s="2">
         <v>18.25</v>
       </c>
     </row>
-    <row r="187" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A187" s="2">
         <v>18.5</v>
       </c>
     </row>
-    <row r="188" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A188" s="2">
         <v>18.75</v>
       </c>
     </row>
-    <row r="189" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A189" s="2">
         <v>19</v>
       </c>
     </row>
-    <row r="190" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A190" s="2">
         <v>19.25</v>
       </c>
     </row>
-    <row r="191" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A191" s="2">
         <v>19.5</v>
       </c>
     </row>
-    <row r="192" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A192" s="2">
         <v>19.75</v>
       </c>
     </row>
-    <row r="193" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A193" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="197" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="198" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="199" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="16" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="200" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="16" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="201" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="16" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="202" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="16" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="203" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="16" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="204" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="16" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="205" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="16" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="206" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="16" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="207" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="16" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="208" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A208" s="17" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="209" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A209" s="17" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="210" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A210" s="16" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="211" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A211" s="16" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="212" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A212" s="16" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="213" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A213" s="16" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="214" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A214" s="16" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="215" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A215" s="16" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="216" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A216" s="16" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="217" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A217" s="16" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="218" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A218" s="16" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="219" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A219" s="16" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="220" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A220" s="16" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="221" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A221" s="16" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="222" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A222" s="16" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="223" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A223" s="16" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="224" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A224" s="16" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="225" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A225" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="226" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A226" s="16" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="227" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A227" s="16" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="228" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A228" s="16" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="229" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A229" s="16" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="230" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A230" s="16" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="231" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A231" s="16" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="232" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A232" s="16" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="233" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A233" s="16" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="234" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A234" s="16" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="235" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A235" s="16" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="236" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A236" s="18" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="237" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A237" s="16" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="238" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A238" s="16" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="239" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A239" s="16" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="240" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A240" s="16" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="241" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A241" s="16" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="242" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A242" s="16" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="243" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A243" s="16" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="244" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A244" s="16" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="245" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A245" s="16" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="246" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A246" s="16" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="247" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A247" s="16" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="248" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A248" s="16" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="249" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A249" s="16" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="250" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A250" s="16" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="251" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A251" s="18" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="252" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A252" s="19" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="253" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A253" s="16" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="254" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A254" s="16" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="255" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A255" s="20" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="256" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A256" s="20" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="257" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A257" s="21" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="258" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A258" s="16" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="259" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A259" s="21" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="260" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A260" s="16" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="261" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A261" s="21" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="262" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A262" s="16" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="263" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A263" s="16" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="264" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A264" s="21" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="265" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A265" s="21" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="266" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A266" s="21" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="267" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A267" s="16" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="268" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A268" s="16" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="269" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A269" s="16" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="270" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A270" s="16" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="271" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A271" s="21" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="272" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A272" s="21" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="273" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A273" s="16" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="274" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A274" s="21" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="275" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A275" s="21" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="276" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A276" s="16" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="277" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A277" s="16" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="278" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A278" s="21" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="279" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A279" s="16" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="280" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A280" s="16" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="281" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A281" s="16" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="282" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A282" s="16" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="283" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A283" s="21" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="284" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A284" s="21" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="285" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A285" s="21" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="286" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A286" s="16" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="287" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A287" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="288" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A288" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="289" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A289" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="290" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A290" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="291" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A291" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="292" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A292" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="293" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A293" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="294" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A294" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="295" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A295" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="296" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A296" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="297" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A297" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="298" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A298" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="299" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A299" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="300" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A300" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="301" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A301" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="302" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A302" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="303" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A303" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="304" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A304" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="305" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A305" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="306" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A306" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="307" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A307" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="308" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A308" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="309" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A309" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="310" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A310" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="311" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A311" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="312" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A312" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="313" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A313" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="314" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A314" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="315" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A315" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="316" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A316" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="317" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A317" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="318" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A318" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="319" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A319" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="320" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A320" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="321" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A321" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="322" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A322" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="323" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A323" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="324" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A324" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="325" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A325" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="326" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A326" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="327" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A327" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="328" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A328" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="329" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A329" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="330" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A330" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="331" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A331" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="332" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A332" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="333" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A333" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="334" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A334" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="335" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A335" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="336" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A336" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="337" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A337" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="338" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A338" s="2" t="s">
         <v>54</v>
       </c>

</xml_diff>